<commit_message>
test: make worksheet print qualification platform independent
</commit_message>
<xml_diff>
--- a/test/fixtures/color-blocks.xlsx
+++ b/test/fixtures/color-blocks.xlsx
@@ -4,6 +4,9 @@
   <sheets>
     <sheet name="Render" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Render!$A$1:$B$2</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -65,6 +68,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B2"/>
   <cols>
     <col min="1" max="2" width="24" customWidth="1"/>
@@ -95,5 +101,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>